<commit_message>
Loretta, Knight of the Haligtree | Add datasheets of microcontrollers to appendix of thesis; Changes in the ESP32-DevKit-C chapter; Add full chapter about Raspberry Pi Pico 2W; Research and compare different microcontrollers; Remove old price comparison images; Adjust formula to rank cost; Adjust image so percentages are correct again; Minor changes in microcontroller chapters
</commit_message>
<xml_diff>
--- a/Diplomarbeit/doc/Schaar/Tabellenberechnungen_Diagramme_Diplomarbeit_Schaar.xlsx
+++ b/Diplomarbeit/doc/Schaar/Tabellenberechnungen_Diagramme_Diplomarbeit_Schaar.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kiese\OneDrive\Dokumente\Schule\Diplomarbeit\Diplomarbeit_Tischkicker\Diplomarbeit\doc\Schaar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3531D81-8E06-439C-AED9-3BEACA226312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46BA01CE-529C-4D61-BA5A-FCEF19F75FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{6E91DB90-8AB8-47FA-9925-F6AA49AB0963}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{6E91DB90-8AB8-47FA-9925-F6AA49AB0963}"/>
   </bookViews>
   <sheets>
     <sheet name="Diagramm - Punkteverteilung MCs" sheetId="1" r:id="rId1"/>
+    <sheet name="Diagramm - Vergleich MCs" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
   <si>
     <t>Vergleichsbasis</t>
   </si>
@@ -60,13 +61,70 @@
   </si>
   <si>
     <t>Gesamt</t>
+  </si>
+  <si>
+    <t>Punktekategorie</t>
+  </si>
+  <si>
+    <t>Punktevergabe - Mikrocontroller</t>
+  </si>
+  <si>
+    <t>Arduino Nano ESP32</t>
+  </si>
+  <si>
+    <t>ESP32 DevKit C</t>
+  </si>
+  <si>
+    <t>Raspberry Pi Pico 2W</t>
+  </si>
+  <si>
+    <t>Preis (in €)</t>
+  </si>
+  <si>
+    <t>https://store.arduino.cc/collections/nano-family/products/nano-esp32-with-headers</t>
+  </si>
+  <si>
+    <t>https://www.mouser.at/ProductDetail/Arduino/ABX00083?qs=ulEaXIWI0c8OkA6u7pnNRA%3D%3D</t>
+  </si>
+  <si>
+    <t>Durchschnittlicher Preis</t>
+  </si>
+  <si>
+    <t>https://www.reichelt.at/at/de/shop/produkt/arduino_nano_esp32_mit_header_esp32-s3_usb-c-353087</t>
+  </si>
+  <si>
+    <t>Händler-Links (mit Kosten/1 St. exkl. Versand) für jeden Mikrocontroller (Stand 18.02.2026)</t>
+  </si>
+  <si>
+    <t>https://shop4akku.de/esp32-devkit-v4/</t>
+  </si>
+  <si>
+    <t>https://www.az-delivery.de/products/esp-32-dev-kit-c-v4</t>
+  </si>
+  <si>
+    <t>https://shop.heise.de/esp-32-dev-kit-c-v4</t>
+  </si>
+  <si>
+    <t>https://www.welectron.com/Raspberry-Pi-Pico-2-W?src=raspberrypi</t>
+  </si>
+  <si>
+    <t>https://www.berrybase.at/raspberry-pi-pico-2w-rp2350-wlan-bluetooth-mikrocontroller-board</t>
+  </si>
+  <si>
+    <t>https://www.reichelt.at/at/de/shop/produkt/raspberry_pi_pico_2_wh_rp235x_cortex-m33_wifi_microusb-398576</t>
+  </si>
+  <si>
+    <t>Gesamtpunktzahl</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,8 +148,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -122,8 +195,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -224,30 +321,211 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="1" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="1" fillId="8" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="1" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="2" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="2" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Link" xfId="2" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Währung" xfId="1" builtinId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -622,16 +900,16 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.6</c:v>
+                  <c:v>0.49</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.17</c:v>
+                  <c:v>0.22</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.17</c:v>
+                  <c:v>0.22</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.06</c:v>
+                  <c:v>7.0000000000000007E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1662,10 +1940,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="6"/>
+      <c r="B1" s="11"/>
     </row>
     <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -1679,39 +1957,39 @@
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7">
-        <v>0.6</v>
+      <c r="B3" s="5">
+        <v>0.49</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="7">
-        <v>0.17</v>
+      <c r="B4" s="5">
+        <v>0.22</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="7">
-        <v>0.17</v>
+      <c r="B5" s="5">
+        <v>0.22</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="9">
-        <v>0.06</v>
+      <c r="B6" s="7">
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="9">
         <f>SUM(B3:B6)</f>
         <v>1</v>
       </c>
@@ -1724,4 +2002,263 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A80091F7-2C5E-465A-85A8-C5C259172273}">
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="100.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="11"/>
+      <c r="F1" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="13"/>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="19">
+        <f>MIN(20, ROUNDUP(100/G6,0))</f>
+        <v>6</v>
+      </c>
+      <c r="C3" s="19">
+        <f>MIN(20, ROUNDUP(100/G12,0))</f>
+        <v>8</v>
+      </c>
+      <c r="D3" s="38">
+        <f>MIN(20, ROUNDUP(100/G18,0))</f>
+        <v>13</v>
+      </c>
+      <c r="F3" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="28">
+        <v>21.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="19">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1">
+        <v>9</v>
+      </c>
+      <c r="D4" s="37">
+        <v>3</v>
+      </c>
+      <c r="F4" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="30">
+        <v>16.600000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="19">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1">
+        <v>3</v>
+      </c>
+      <c r="D5" s="37">
+        <v>9</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="30">
+        <v>19.97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="20">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1">
+        <v>6</v>
+      </c>
+      <c r="D6" s="37">
+        <v>9</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="23">
+        <f>AVERAGE(G3:G5)</f>
+        <v>19.39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="36">
+        <f>SUM(B3:B6)</f>
+        <v>21</v>
+      </c>
+      <c r="C7" s="35">
+        <f t="shared" ref="C7:D7" si="0">SUM(C3:C6)</f>
+        <v>26</v>
+      </c>
+      <c r="D7" s="35">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="F7" s="33"/>
+      <c r="G7" s="34"/>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F8" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F9" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="28">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F10" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="30">
+        <v>13.99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F11" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="30">
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F12" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="26">
+        <f>AVERAGE(G9:G11)</f>
+        <v>12.963333333333333</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F13" s="33"/>
+      <c r="G13" s="34"/>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F14" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F15" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="G15" s="30">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F16" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="30">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="6:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F17" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" s="30">
+        <v>8.57</v>
+      </c>
+    </row>
+    <row r="18" spans="6:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F18" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="25">
+        <f>AVERAGE(G15:G17)</f>
+        <v>8.0566666666666666</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="F1:G1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="F3" r:id="rId1" xr:uid="{BDA6AC5D-0BB1-4150-A48B-314E56DBAE5E}"/>
+    <hyperlink ref="F4" r:id="rId2" xr:uid="{EEAD633B-863E-41E1-ABC0-07CD316DE6C1}"/>
+    <hyperlink ref="F5" r:id="rId3" xr:uid="{B8565D1B-4D94-4C34-801E-47129249B15B}"/>
+    <hyperlink ref="F9" r:id="rId4" xr:uid="{9A5D1B25-1B18-4807-8E9B-D6D5BF88BB30}"/>
+    <hyperlink ref="F10" r:id="rId5" xr:uid="{37BDFEF7-3837-45A9-BCA3-43E81D9197A4}"/>
+    <hyperlink ref="F11" r:id="rId6" xr:uid="{FED469AC-0385-4F1F-8623-34354F0D1BB7}"/>
+    <hyperlink ref="F15" r:id="rId7" xr:uid="{E5690637-2148-484E-BA59-046FE1C0F873}"/>
+    <hyperlink ref="F16" r:id="rId8" xr:uid="{801DEA99-48F7-4380-B225-1DF58CCF9D6D}"/>
+    <hyperlink ref="F17" r:id="rId9" xr:uid="{1FC1C8E0-D738-4D70-9366-DE5FDD63D7C8}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ulcerated Tree Spirit | Fix minor mistakes in thesis; Add captions to code segments for proper rendering; Remove duplicate .pdf files from doc directory as well as temporary .pptx file; Add table calculations to appendix of thesis; Add diagrams as images for data visualization; Remove unused/dummy files from pdfs directory (except 1 to test proper appendix rendering); Write chapter about comparison of microcontroller options; Move the chapter 'Creation of instructions for reproduction' to practical part of the thesis, since it isn't theoretical work
</commit_message>
<xml_diff>
--- a/Diplomarbeit/doc/Schaar/Tabellenberechnungen_Diagramme_Diplomarbeit_Schaar.xlsx
+++ b/Diplomarbeit/doc/Schaar/Tabellenberechnungen_Diagramme_Diplomarbeit_Schaar.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kiese\OneDrive\Dokumente\Schule\Diplomarbeit\Diplomarbeit_Tischkicker\Diplomarbeit\doc\Schaar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46BA01CE-529C-4D61-BA5A-FCEF19F75FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2637B0D-283B-44CF-829A-9101ACDD01F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{6E91DB90-8AB8-47FA-9925-F6AA49AB0963}"/>
   </bookViews>
   <sheets>
     <sheet name="Diagramm - Punkteverteilung MCs" sheetId="1" r:id="rId1"/>
-    <sheet name="Diagramm - Vergleich MCs" sheetId="2" r:id="rId2"/>
+    <sheet name="Berechnung - Vergleich MCs" sheetId="2" r:id="rId2"/>
+    <sheet name="Diagramm - Vergleich MCs" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -121,10 +122,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_-&quot;€&quot;\ * #,##0.00_-;\-&quot;€&quot;\ * #,##0.00_-;_-&quot;€&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="&quot;€&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +161,29 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -220,7 +245,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -322,7 +347,173 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right/>
@@ -333,9 +524,7 @@
     <border>
       <left/>
       <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -345,52 +534,6 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
@@ -398,71 +541,6 @@
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -471,7 +549,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -482,45 +560,131 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="1" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="1" fillId="8" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="1" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="2" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="2" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="2" builtinId="8"/>
@@ -1015,7 +1179,937 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="95000"/>
+                    <a:lumOff val="5000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="de-AT"/>
+              <a:t>Punkteverteilung - Mikrocontroller</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="95000"/>
+                  <a:lumOff val="5000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-AT"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Berechnung - Vergleich MCs'!$B$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Arduino Nano ESP32</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Berechnung - Vergleich MCs'!$A$3:$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Kosten</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Prozessorleistung</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Datenübertragung</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Stromverbrauch</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Berechnung - Vergleich MCs'!$B$3:$B$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A35F-4826-A638-DFF1E37CA8F9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Berechnung - Vergleich MCs'!$C$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ESP32 DevKit C</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Berechnung - Vergleich MCs'!$A$3:$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Kosten</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Prozessorleistung</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Datenübertragung</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Stromverbrauch</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Berechnung - Vergleich MCs'!$C$3:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-A35F-4826-A638-DFF1E37CA8F9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Berechnung - Vergleich MCs'!$D$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Raspberry Pi Pico 2W</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Berechnung - Vergleich MCs'!$A$3:$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Kosten</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Prozessorleistung</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Datenübertragung</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Stromverbrauch</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Berechnung - Vergleich MCs'!$D$3:$D$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-A35F-4826-A638-DFF1E37CA8F9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="960533439"/>
+        <c:axId val="960534399"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="960533439"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1050" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="95000"/>
+                    <a:lumOff val="5000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="960534399"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="960534399"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="95000"/>
+                    <a:lumOff val="5000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="960533439"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="95000"/>
+                  <a:lumOff val="5000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:solidFill>
+            <a:schemeClr val="tx1">
+              <a:lumMod val="95000"/>
+              <a:lumOff val="5000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+          <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.7" r="0.7" t="0.78740157499999996" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="95000"/>
+                    <a:lumOff val="5000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="de-AT"/>
+              <a:t>Gesamtpunktzahl - Mikrocontroller</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="95000"/>
+                  <a:lumOff val="5000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-AT"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-8E1F-4E01-9A63-70A89FF1BDFB}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-8E1F-4E01-9A63-70A89FF1BDFB}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Berechnung - Vergleich MCs'!$B$2:$D$2</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Arduino Nano ESP32</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>ESP32 DevKit C</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Raspberry Pi Pico 2W</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Berechnung - Vergleich MCs'!$B$7:$D$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>28</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8E1F-4E01-9A63-70A89FF1BDFB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="1023529951"/>
+        <c:axId val="1023533791"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1023529951"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="95000"/>
+                    <a:lumOff val="5000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1023533791"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1023533791"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="95000"/>
+                    <a:lumOff val="5000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1023529951"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:solidFill>
+            <a:schemeClr val="tx1">
+              <a:lumMod val="95000"/>
+              <a:lumOff val="5000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:latin typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+          <a:cs typeface="72 Monospace" panose="020B0509030603020204" pitchFamily="49" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.7" r="0.7" t="0.78740157499999996" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1574,6 +2668,1014 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1607,6 +3709,87 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>104774</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>9524</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>114299</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>53339</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Diagramm 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{164BCEB3-10C7-40FF-B317-95576B4F5D91}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>95249</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>57149</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>111124</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>104774</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Diagramm 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4AA50F57-F6F9-4D9C-B154-887E06F03BFF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1940,10 +4123,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="11"/>
+      <c r="B1" s="33"/>
     </row>
     <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -2006,13 +4189,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A80091F7-2C5E-465A-85A8-C5C259172273}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="52.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
     <col min="6" max="6" width="100.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
@@ -2021,244 +4204,322 @@
     <col min="12" max="12" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:4" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="11"/>
-      <c r="F1" s="12" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="36"/>
+    </row>
+    <row r="2" spans="1:4" ht="38.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="20">
+        <f>MIN(20, ROUNDUP(100/B15,0))</f>
+        <v>6</v>
+      </c>
+      <c r="C3" s="20">
+        <f>MIN(20, ROUNDUP(100/B21,0))</f>
+        <v>8</v>
+      </c>
+      <c r="D3" s="21">
+        <f>MIN(20, ROUNDUP(100/B27,0))</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="20">
+        <v>6</v>
+      </c>
+      <c r="C4" s="23">
+        <v>9</v>
+      </c>
+      <c r="D4" s="24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="20">
+        <v>6</v>
+      </c>
+      <c r="C5" s="23">
+        <v>3</v>
+      </c>
+      <c r="D5" s="24">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="25">
+        <v>1</v>
+      </c>
+      <c r="C6" s="23">
+        <v>2</v>
+      </c>
+      <c r="D6" s="24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="27">
+        <f>SUM(B3:B6)</f>
+        <v>19</v>
+      </c>
+      <c r="C7" s="28">
+        <f t="shared" ref="C7:D7" si="0">SUM(C3:C6)</f>
+        <v>22</v>
+      </c>
+      <c r="D7" s="28">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="13"/>
+      <c r="B10" s="38"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="39"/>
     </row>
-    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+    <row r="11" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="41"/>
+      <c r="D11" s="42"/>
+    </row>
+    <row r="12" spans="1:4" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="43">
+        <v>21.6</v>
+      </c>
+      <c r="C12" s="44"/>
+      <c r="D12" s="45"/>
+    </row>
+    <row r="13" spans="1:4" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="43">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="C13" s="44"/>
+      <c r="D13" s="45"/>
+    </row>
+    <row r="14" spans="1:4" ht="31.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="43">
+        <v>19.97</v>
+      </c>
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+    </row>
+    <row r="15" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="46">
+        <f>AVERAGE(B12:B14)</f>
+        <v>19.39</v>
+      </c>
+      <c r="C15" s="47"/>
+      <c r="D15" s="48"/>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="17"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="50"/>
+    </row>
+    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="52"/>
+      <c r="D17" s="53"/>
+    </row>
+    <row r="18" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A18" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="43">
+        <v>13</v>
+      </c>
+      <c r="C18" s="44"/>
+      <c r="D18" s="45"/>
+    </row>
+    <row r="19" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="43">
+        <v>13.99</v>
+      </c>
+      <c r="C19" s="44"/>
+      <c r="D19" s="45"/>
+    </row>
+    <row r="20" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="43">
+        <v>11.9</v>
+      </c>
+      <c r="C20" s="44"/>
+      <c r="D20" s="45"/>
+    </row>
+    <row r="21" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="57">
+        <f>AVERAGE(B18:B20)</f>
+        <v>12.963333333333333</v>
+      </c>
+      <c r="C21" s="58"/>
+      <c r="D21" s="59"/>
+    </row>
+    <row r="22" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="17"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="50"/>
+    </row>
+    <row r="23" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="61"/>
+      <c r="D23" s="62"/>
+    </row>
+    <row r="24" spans="1:4" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="A24" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="43">
+        <v>7.6</v>
+      </c>
+      <c r="C24" s="44"/>
+      <c r="D24" s="45"/>
+    </row>
+    <row r="25" spans="1:4" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="43">
         <v>8</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>13</v>
-      </c>
+      <c r="C25" s="44"/>
+      <c r="D25" s="45"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="19">
-        <f>MIN(20, ROUNDUP(100/G6,0))</f>
-        <v>6</v>
-      </c>
-      <c r="C3" s="19">
-        <f>MIN(20, ROUNDUP(100/G12,0))</f>
-        <v>8</v>
-      </c>
-      <c r="D3" s="38">
-        <f>MIN(20, ROUNDUP(100/G18,0))</f>
-        <v>13</v>
-      </c>
-      <c r="F3" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="28">
-        <v>21.6</v>
-      </c>
+    <row r="26" spans="1:4" ht="31.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="43">
+        <v>8.57</v>
+      </c>
+      <c r="C26" s="44"/>
+      <c r="D26" s="45"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="19">
-        <v>6</v>
-      </c>
-      <c r="C4" s="1">
-        <v>9</v>
-      </c>
-      <c r="D4" s="37">
-        <v>3</v>
-      </c>
-      <c r="F4" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="30">
-        <v>16.600000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="31" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="19">
-        <v>6</v>
-      </c>
-      <c r="C5" s="1">
-        <v>3</v>
-      </c>
-      <c r="D5" s="37">
-        <v>9</v>
-      </c>
-      <c r="F5" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="30">
-        <v>19.97</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="31" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="20">
-        <v>3</v>
-      </c>
-      <c r="C6" s="1">
-        <v>6</v>
-      </c>
-      <c r="D6" s="37">
-        <v>9</v>
-      </c>
-      <c r="F6" s="4" t="s">
+    <row r="27" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="23">
-        <f>AVERAGE(G3:G5)</f>
-        <v>19.39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="36">
-        <f>SUM(B3:B6)</f>
-        <v>21</v>
-      </c>
-      <c r="C7" s="35">
-        <f t="shared" ref="C7:D7" si="0">SUM(C3:C6)</f>
-        <v>26</v>
-      </c>
-      <c r="D7" s="35">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-      <c r="F7" s="33"/>
-      <c r="G7" s="34"/>
-    </row>
-    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F8" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F9" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="28">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F10" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="30">
-        <v>13.99</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F11" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" s="30">
-        <v>11.9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F12" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="G12" s="26">
-        <f>AVERAGE(G9:G11)</f>
-        <v>12.963333333333333</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F13" s="33"/>
-      <c r="G13" s="34"/>
-    </row>
-    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F14" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="21" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F15" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="G15" s="30">
-        <v>7.6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F16" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="G16" s="30">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="6:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F17" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="G17" s="30">
-        <v>8.57</v>
-      </c>
-    </row>
-    <row r="18" spans="6:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F18" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="G18" s="25">
-        <f>AVERAGE(G15:G17)</f>
+      <c r="B27" s="54">
+        <f>AVERAGE(B24:B26)</f>
         <v>8.0566666666666666</v>
       </c>
+      <c r="C27" s="55"/>
+      <c r="D27" s="56"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="19">
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="F3" r:id="rId1" xr:uid="{BDA6AC5D-0BB1-4150-A48B-314E56DBAE5E}"/>
-    <hyperlink ref="F4" r:id="rId2" xr:uid="{EEAD633B-863E-41E1-ABC0-07CD316DE6C1}"/>
-    <hyperlink ref="F5" r:id="rId3" xr:uid="{B8565D1B-4D94-4C34-801E-47129249B15B}"/>
-    <hyperlink ref="F9" r:id="rId4" xr:uid="{9A5D1B25-1B18-4807-8E9B-D6D5BF88BB30}"/>
-    <hyperlink ref="F10" r:id="rId5" xr:uid="{37BDFEF7-3837-45A9-BCA3-43E81D9197A4}"/>
-    <hyperlink ref="F11" r:id="rId6" xr:uid="{FED469AC-0385-4F1F-8623-34354F0D1BB7}"/>
-    <hyperlink ref="F15" r:id="rId7" xr:uid="{E5690637-2148-484E-BA59-046FE1C0F873}"/>
-    <hyperlink ref="F16" r:id="rId8" xr:uid="{801DEA99-48F7-4380-B225-1DF58CCF9D6D}"/>
-    <hyperlink ref="F17" r:id="rId9" xr:uid="{1FC1C8E0-D738-4D70-9366-DE5FDD63D7C8}"/>
+    <hyperlink ref="A12" r:id="rId1" xr:uid="{BDA6AC5D-0BB1-4150-A48B-314E56DBAE5E}"/>
+    <hyperlink ref="A13" r:id="rId2" xr:uid="{EEAD633B-863E-41E1-ABC0-07CD316DE6C1}"/>
+    <hyperlink ref="A14" r:id="rId3" xr:uid="{B8565D1B-4D94-4C34-801E-47129249B15B}"/>
+    <hyperlink ref="A18" r:id="rId4" xr:uid="{9A5D1B25-1B18-4807-8E9B-D6D5BF88BB30}"/>
+    <hyperlink ref="A19" r:id="rId5" xr:uid="{37BDFEF7-3837-45A9-BCA3-43E81D9197A4}"/>
+    <hyperlink ref="A20" r:id="rId6" xr:uid="{FED469AC-0385-4F1F-8623-34354F0D1BB7}"/>
+    <hyperlink ref="A24" r:id="rId7" xr:uid="{E5690637-2148-484E-BA59-046FE1C0F873}"/>
+    <hyperlink ref="A25" r:id="rId8" xr:uid="{801DEA99-48F7-4380-B225-1DF58CCF9D6D}"/>
+    <hyperlink ref="A26" r:id="rId9" xr:uid="{1FC1C8E0-D738-4D70-9366-DE5FDD63D7C8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DFDEF53-5A19-4925-A325-77AB2F0E6D99}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>